<commit_message>
added more stop pd reason and added some episode type scenarios
</commit_message>
<xml_diff>
--- a/inst/extdata/pe_2025.xlsx
+++ b/inst/extdata/pe_2025.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -421,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -867,6 +868,210 @@
         <v>45990</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SPD0003</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>45731</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Staphylococcus epidermidis</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>45745</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SPD0018</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>45826</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Klebsiella pneumoniae</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>45840</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SPD0033</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>45879</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Staphylococcus aureus</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>45893</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SPD0023</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>45783</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>45797</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SPD0030</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>45950</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Pseudomonas aeruginosa</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>45964</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SPD0046</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>45910</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Staphylococcus aureus</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>45924</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SPD0046</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>45945</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Pseudomonas aeruginosa</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>45959</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SPD0047</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>45971</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>45985</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SPD0041</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>45848</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Escherichia coli</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>45862</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SPD0012</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>45920</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Staphylococcus aureus</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>45934</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>